<commit_message>
Update SMS campaign targets (add VIP/サンクス/バースデー, latest 11 types)
</commit_message>
<xml_diff>
--- a/SMSターゲット.xlsx
+++ b/SMSターゲット.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Media01C/Desktop/Claude IN PROGRESS/【P】SMS分析レポート作成/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED66498F-309A-EE42-BB03-D860F4287D75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D15ABF-1938-7247-9EE1-2B18E52C52E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41220" yWindow="7560" windowWidth="27560" windowHeight="16360" xr2:uid="{95BEBC37-EFA6-B44E-84D0-8D1D2EDFA09E}"/>
+    <workbookView xWindow="41800" yWindow="500" windowWidth="15480" windowHeight="16160" xr2:uid="{95BEBC37-EFA6-B44E-84D0-8D1D2EDFA09E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,144 +39,72 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+  <si>
+    <t>1ヶ月未満</t>
+  </si>
+  <si>
+    <t>2〜3ヶ月</t>
+  </si>
+  <si>
+    <t>3〜6ヶ月</t>
+  </si>
+  <si>
+    <t>半年〜1年</t>
+  </si>
+  <si>
+    <t>1〜3年</t>
+  </si>
+  <si>
+    <t>内容</t>
+  </si>
+  <si>
+    <t>ターゲット離反会員期間</t>
+  </si>
+  <si>
+    <t>備考</t>
+  </si>
   <si>
     <t>一般的な新台入替</t>
-    <rPh sb="0" eb="3">
-      <t xml:space="preserve">イッパンテキナ </t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t xml:space="preserve">シンダイ </t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t xml:space="preserve">イレカエ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>大型新台入替</t>
-    <rPh sb="0" eb="2">
-      <t xml:space="preserve">オオガタ </t>
-    </rPh>
-    <rPh sb="2" eb="6">
-      <t xml:space="preserve">シンダイイレカエ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>BIGタイトル新台入替</t>
   </si>
   <si>
     <t>リニューアルオープン</t>
-    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>月間スケジュール案内</t>
   </si>
   <si>
     <t>大型連休スケジュール案内</t>
-    <rPh sb="0" eb="1">
-      <t xml:space="preserve">オオガタ </t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t xml:space="preserve">レンキュウ </t>
-    </rPh>
-    <rPh sb="10" eb="12">
-      <t xml:space="preserve">アンナイ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>月間スケジュール案内</t>
-    <rPh sb="0" eb="2">
-      <t xml:space="preserve">ゲッカン </t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t xml:space="preserve">アンナイ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>特日</t>
+  </si>
+  <si>
+    <t>年一の特日案内</t>
   </si>
   <si>
     <t>入会サンクス</t>
-    <rPh sb="0" eb="2">
-      <t xml:space="preserve">ニュウカイ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>内容</t>
-    <rPh sb="0" eb="2">
-      <t xml:space="preserve">ナイヨウ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>バースデー</t>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>月に一度の案内なので、対象者は12分の1に下げる</t>
-    <rPh sb="0" eb="1">
-      <t xml:space="preserve">ツキニ </t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t xml:space="preserve">イチド </t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t xml:space="preserve">アンナイ </t>
-    </rPh>
-    <rPh sb="11" eb="14">
-      <t xml:space="preserve">タイショウシャ </t>
-    </rPh>
-    <rPh sb="17" eb="18">
-      <t xml:space="preserve">ブン </t>
-    </rPh>
-    <rPh sb="21" eb="22">
-      <t xml:space="preserve">サゲル </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>BIGタイトル新台入替</t>
-    <rPh sb="7" eb="9">
-      <t xml:space="preserve">シンダイ </t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t xml:space="preserve">イレカエ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>1ヶ月未満</t>
-  </si>
-  <si>
-    <t>2〜3ヶ月</t>
-  </si>
-  <si>
-    <t>3〜6ヶ月</t>
-  </si>
-  <si>
-    <t>半年〜1年</t>
-  </si>
-  <si>
-    <t>1〜3年</t>
-  </si>
-  <si>
-    <t>ターゲット離反会員期間</t>
-    <rPh sb="5" eb="9">
-      <t xml:space="preserve">リハンカイインソウ </t>
-    </rPh>
-    <rPh sb="9" eb="11">
-      <t xml:space="preserve">キカン </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>備考</t>
-    <rPh sb="0" eb="2">
-      <t xml:space="preserve">ビコウ </t>
-    </rPh>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>VIP会員</t>
-    <rPh sb="3" eb="5">
-      <t xml:space="preserve">カイイン </t>
-    </rPh>
+  </si>
+  <si>
+    <t>台数の20%にする</t>
+  </si>
+  <si>
+    <t>台数の10%にする</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -184,7 +112,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -199,24 +127,25 @@
       <charset val="128"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Meiryo"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF27272A"/>
+      <color rgb="FF333333"/>
       <name val="Yu Gothic UI"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -252,13 +181,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -595,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D4AD3B0-CA6E-9B47-9992-84AB92572F18}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="20" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -605,97 +534,119 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="2"/>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>

</xml_diff>